<commit_message>
fix: skip blank experiment rows and add RDA no-share group
</commit_message>
<xml_diff>
--- a/a.输入/批量实验配置.xlsx
+++ b/a.输入/批量实验配置.xlsx
@@ -2719,7 +2719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col width="33.1428571428571" customWidth="1" min="1" max="1"/>
@@ -2892,6 +2892,7 @@
         <v>1</v>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -2964,6 +2965,14 @@
         <v>1</v>
       </c>
     </row>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
@@ -3322,6 +3331,42 @@
       </c>
       <c r="J25" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>RDA</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Without share weighting</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>5</v>
+      </c>
+      <c r="D26" t="n">
+        <v>5</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" t="n">
+        <v>2</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="n">
+        <v>1</v>
+      </c>
+      <c r="J26" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>